<commit_message>
Removes outdated spreadsheet and updates related files
Deletes an obsolete file to streamline resources and updates
two spreadsheets with revised content or structure to ensure
data remains current and relevant.
</commit_message>
<xml_diff>
--- a/excel/day_routine.xlsx
+++ b/excel/day_routine.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
   <si>
     <t>Time</t>
   </si>
@@ -79,21 +80,12 @@
     <t>Optional</t>
   </si>
   <si>
-    <t>1-hour duration</t>
-  </si>
-  <si>
     <t>45 minutes</t>
   </si>
   <si>
-    <t>Before this time</t>
-  </si>
-  <si>
     <t>Wake up / Drink 2 glasses of water / Make Bed</t>
   </si>
   <si>
-    <t>Physical Activity</t>
-  </si>
-  <si>
     <t>Skin Care, Hair care</t>
   </si>
   <si>
@@ -121,18 +113,6 @@
     <t>8:45 AM</t>
   </si>
   <si>
-    <t>7:45 AM</t>
-  </si>
-  <si>
-    <t>7:30 AM</t>
-  </si>
-  <si>
-    <t>7:00 AM</t>
-  </si>
-  <si>
-    <t>6:00 AM</t>
-  </si>
-  <si>
     <t>5:40 AM</t>
   </si>
   <si>
@@ -146,6 +126,24 @@
   </si>
   <si>
     <t>4:55 AM</t>
+  </si>
+  <si>
+    <t>Jogging</t>
+  </si>
+  <si>
+    <t>6:40 AM</t>
+  </si>
+  <si>
+    <t>7:40 AM</t>
+  </si>
+  <si>
+    <t>8:10 AM</t>
+  </si>
+  <si>
+    <t>8:25 AM</t>
+  </si>
+  <si>
+    <t>Before 11.00 pm</t>
   </si>
 </sst>
 </file>
@@ -553,16 +551,16 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="4" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="5" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>7</v>
@@ -571,7 +569,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>8</v>
@@ -580,7 +578,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="5" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>6</v>
@@ -589,10 +587,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="5" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="C6" s="2"/>
     </row>
@@ -612,12 +610,12 @@
         <v>38</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>10</v>
@@ -626,27 +624,25 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="5" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
@@ -667,13 +663,13 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -696,16 +692,16 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>17</v>
@@ -714,7 +710,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>18</v>
@@ -723,16 +719,25 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updates Excel files with revised data
Incorporates new information or adjustments to planning spreadsheets,
ensuring more accurate and up-to-date tracking for daily routines and
weight loss planning.
</commit_message>
<xml_diff>
--- a/excel/day_routine.xlsx
+++ b/excel/day_routine.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Time</t>
   </si>
@@ -23,9 +23,6 @@
     <t>Task</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>2:00 PM</t>
   </si>
   <si>
@@ -35,18 +32,6 @@
     <t>4:15 PM</t>
   </si>
   <si>
-    <t>Sit silently and deep breathe</t>
-  </si>
-  <si>
-    <t>Restroom and track weight</t>
-  </si>
-  <si>
-    <t>Oil pulling and brushing</t>
-  </si>
-  <si>
-    <t>If needed: Self-care</t>
-  </si>
-  <si>
     <t>Prepare breakfast and eat</t>
   </si>
   <si>
@@ -74,24 +59,6 @@
     <t>Prepare for sleep</t>
   </si>
   <si>
-    <t>Sleep</t>
-  </si>
-  <si>
-    <t>Optional</t>
-  </si>
-  <si>
-    <t>45 minutes</t>
-  </si>
-  <si>
-    <t>Wake up / Drink 2 glasses of water / Make Bed</t>
-  </si>
-  <si>
-    <t>Skin Care, Hair care</t>
-  </si>
-  <si>
-    <t>Pre Skincare, Hair Care and Bathing</t>
-  </si>
-  <si>
     <t>Come back, fresh up, and prepare rice</t>
   </si>
   <si>
@@ -110,18 +77,6 @@
     <t>3:00 PM</t>
   </si>
   <si>
-    <t>8:45 AM</t>
-  </si>
-  <si>
-    <t>5:40 AM</t>
-  </si>
-  <si>
-    <t>5:20 AM</t>
-  </si>
-  <si>
-    <t>5:35 AM</t>
-  </si>
-  <si>
     <t>5:05 AM</t>
   </si>
   <si>
@@ -131,19 +86,49 @@
     <t>Jogging</t>
   </si>
   <si>
-    <t>6:40 AM</t>
-  </si>
-  <si>
-    <t>7:40 AM</t>
-  </si>
-  <si>
-    <t>8:10 AM</t>
-  </si>
-  <si>
-    <t>8:25 AM</t>
-  </si>
-  <si>
-    <t>Before 11.00 pm</t>
+    <t>5.00 AM</t>
+  </si>
+  <si>
+    <t>Wake up</t>
+  </si>
+  <si>
+    <t>Track weight / Drink 2 glasses of water</t>
+  </si>
+  <si>
+    <t>Get ready for the Jogging</t>
+  </si>
+  <si>
+    <t>5:10 AM</t>
+  </si>
+  <si>
+    <t>Oil Pulling / Brushing</t>
+  </si>
+  <si>
+    <t>6:10 AM</t>
+  </si>
+  <si>
+    <t>Stretch</t>
+  </si>
+  <si>
+    <t>6:20 AM</t>
+  </si>
+  <si>
+    <t>6.35 AM</t>
+  </si>
+  <si>
+    <t>7:00 AM</t>
+  </si>
+  <si>
+    <t>Self Care and Fresh up</t>
+  </si>
+  <si>
+    <t>8.45 AM</t>
+  </si>
+  <si>
+    <t>8:15 AM</t>
+  </si>
+  <si>
+    <t>Meditation Before Sleep (Before 11.00 pm)</t>
   </si>
 </sst>
 </file>
@@ -530,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -545,188 +530,170 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="4" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="5" t="s">
-        <v>35</v>
+      <c r="A3" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2"/>
+        <v>25</v>
+      </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="5" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>37</v>
+        <v>29</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>20</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>24</v>
+        <v>32</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="2"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="5" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="A12" s="5"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" s="2"/>
+      <c r="A13" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="5" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="5" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="5" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="5" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="C20" s="2"/>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="2"/>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>42</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>